<commit_message>
dezhurstva: Davydova removed; text size follows the phone setting
Davydova is gone from the doctors, the November order, the Excel file
and the calendars (cal/davydova.ics deleted; build.py now removes
calendars of doctors who are no longer listed). data/config.json gets
an «exclude» list: import_xlsx.py skips those rows in future files and
compose.py never schedules them.

The app's text now scales with the phone's text size: on iPhone the
Dynamic Type body size (-apple-system-body, 17 px by default) sets the
root size, clamped to 0.85–1.5×, and is re-read when the app comes
back to the foreground; Android gets the text-scale meta tag. In «Мои»
the day type moved under the shift time so nothing splits at large
sizes. The test fakes a larger iPhone text size and checks every tab
at ten widths with text 1.15× and 1.4× larger.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D6usDifFMPHewh45USjthA
</commit_message>
<xml_diff>
--- a/dezhurstva/files/2026-11.xlsx
+++ b/dezhurstva/files/2026-11.xlsx
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AF13"/>
+  <dimension ref="A1:AF12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1278,7 +1278,7 @@
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>ДАВЫДОВА</t>
+          <t>ОМУТОВ</t>
         </is>
       </c>
       <c r="B11" s="10" t="n"/>
@@ -1288,9 +1288,17 @@
       <c r="F11" s="11" t="n"/>
       <c r="G11" s="11" t="n"/>
       <c r="H11" s="10" t="n"/>
-      <c r="I11" s="10" t="n"/>
+      <c r="I11" s="10" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="J11" s="11" t="n"/>
-      <c r="K11" s="11" t="n"/>
+      <c r="K11" s="11" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="L11" s="11" t="n"/>
       <c r="M11" s="11" t="n"/>
       <c r="N11" s="11" t="n"/>
@@ -1298,217 +1306,168 @@
       <c r="P11" s="10" t="n"/>
       <c r="Q11" s="11" t="n"/>
       <c r="R11" s="11" t="n"/>
-      <c r="S11" s="11" t="n"/>
+      <c r="S11" s="11" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="T11" s="11" t="n"/>
       <c r="U11" s="11" t="n"/>
       <c r="V11" s="10" t="n"/>
       <c r="W11" s="10" t="n"/>
-      <c r="X11" s="11" t="n"/>
+      <c r="X11" s="11" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="Y11" s="11" t="n"/>
       <c r="Z11" s="11" t="n"/>
       <c r="AA11" s="11" t="n"/>
       <c r="AB11" s="11" t="n"/>
-      <c r="AC11" s="10" t="n"/>
+      <c r="AC11" s="10" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="AD11" s="10" t="n"/>
       <c r="AE11" s="11" t="n"/>
       <c r="AF11" s="12">
         <f>COUNTIF(B11:AE11,"+")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>ОМУТОВ</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="n"/>
-      <c r="C12" s="14" t="n"/>
-      <c r="D12" s="14" t="n"/>
-      <c r="E12" s="10" t="n"/>
-      <c r="F12" s="14" t="n"/>
-      <c r="G12" s="14" t="n"/>
-      <c r="H12" s="10" t="n"/>
-      <c r="I12" s="10" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="J12" s="14" t="n"/>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="L12" s="14" t="n"/>
-      <c r="M12" s="14" t="n"/>
-      <c r="N12" s="14" t="n"/>
-      <c r="O12" s="10" t="n"/>
-      <c r="P12" s="10" t="n"/>
-      <c r="Q12" s="14" t="n"/>
-      <c r="R12" s="14" t="n"/>
-      <c r="S12" s="14" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="T12" s="14" t="n"/>
-      <c r="U12" s="14" t="n"/>
-      <c r="V12" s="10" t="n"/>
-      <c r="W12" s="10" t="n"/>
-      <c r="X12" s="14" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="Y12" s="14" t="n"/>
-      <c r="Z12" s="14" t="n"/>
-      <c r="AA12" s="14" t="n"/>
-      <c r="AB12" s="14" t="n"/>
-      <c r="AC12" s="10" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="AD12" s="10" t="n"/>
-      <c r="AE12" s="14" t="n"/>
-      <c r="AF12" s="12">
-        <f>COUNTIF(B12:AE12,"+")</f>
-        <v>5</v>
+    <row r="12" ht="23" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>Дежурных за день</t>
+        </is>
+      </c>
+      <c r="B12" s="18">
+        <f>COUNTIF(B5:B11,"+")</f>
+        <v>1</v>
+      </c>
+      <c r="C12" s="18">
+        <f>COUNTIF(C5:C11,"+")</f>
+        <v>1</v>
+      </c>
+      <c r="D12" s="18">
+        <f>COUNTIF(D5:D11,"+")</f>
+        <v>1</v>
+      </c>
+      <c r="E12" s="18">
+        <f>COUNTIF(E5:E11,"+")</f>
+        <v>1</v>
+      </c>
+      <c r="F12" s="18">
+        <f>COUNTIF(F5:F11,"+")</f>
+        <v>1</v>
+      </c>
+      <c r="G12" s="18">
+        <f>COUNTIF(G5:G11,"+")</f>
+        <v>1</v>
+      </c>
+      <c r="H12" s="18">
+        <f>COUNTIF(H5:H11,"+")</f>
+        <v>1</v>
+      </c>
+      <c r="I12" s="18">
+        <f>COUNTIF(I5:I11,"+")</f>
+        <v>1</v>
+      </c>
+      <c r="J12" s="18">
+        <f>COUNTIF(J5:J11,"+")</f>
+        <v>1</v>
+      </c>
+      <c r="K12" s="18">
+        <f>COUNTIF(K5:K11,"+")</f>
+        <v>1</v>
+      </c>
+      <c r="L12" s="18">
+        <f>COUNTIF(L5:L11,"+")</f>
+        <v>1</v>
+      </c>
+      <c r="M12" s="18">
+        <f>COUNTIF(M5:M11,"+")</f>
+        <v>1</v>
+      </c>
+      <c r="N12" s="18">
+        <f>COUNTIF(N5:N11,"+")</f>
+        <v>1</v>
+      </c>
+      <c r="O12" s="18">
+        <f>COUNTIF(O5:O11,"+")</f>
+        <v>1</v>
+      </c>
+      <c r="P12" s="18">
+        <f>COUNTIF(P5:P11,"+")</f>
+        <v>1</v>
+      </c>
+      <c r="Q12" s="18">
+        <f>COUNTIF(Q5:Q11,"+")</f>
+        <v>1</v>
+      </c>
+      <c r="R12" s="18">
+        <f>COUNTIF(R5:R11,"+")</f>
+        <v>1</v>
+      </c>
+      <c r="S12" s="18">
+        <f>COUNTIF(S5:S11,"+")</f>
+        <v>1</v>
+      </c>
+      <c r="T12" s="18">
+        <f>COUNTIF(T5:T11,"+")</f>
+        <v>1</v>
+      </c>
+      <c r="U12" s="18">
+        <f>COUNTIF(U5:U11,"+")</f>
+        <v>1</v>
+      </c>
+      <c r="V12" s="18">
+        <f>COUNTIF(V5:V11,"+")</f>
+        <v>1</v>
+      </c>
+      <c r="W12" s="18">
+        <f>COUNTIF(W5:W11,"+")</f>
+        <v>1</v>
+      </c>
+      <c r="X12" s="18">
+        <f>COUNTIF(X5:X11,"+")</f>
+        <v>1</v>
+      </c>
+      <c r="Y12" s="18">
+        <f>COUNTIF(Y5:Y11,"+")</f>
+        <v>1</v>
+      </c>
+      <c r="Z12" s="18">
+        <f>COUNTIF(Z5:Z11,"+")</f>
+        <v>1</v>
+      </c>
+      <c r="AA12" s="18">
+        <f>COUNTIF(AA5:AA11,"+")</f>
+        <v>1</v>
+      </c>
+      <c r="AB12" s="18">
+        <f>COUNTIF(AB5:AB11,"+")</f>
+        <v>1</v>
+      </c>
+      <c r="AC12" s="18">
+        <f>COUNTIF(AC5:AC11,"+")</f>
+        <v>1</v>
+      </c>
+      <c r="AD12" s="18">
+        <f>COUNTIF(AD5:AD11,"+")</f>
+        <v>1</v>
+      </c>
+      <c r="AE12" s="18">
+        <f>COUNTIF(AE5:AE11,"+")</f>
+        <v>1</v>
+      </c>
+      <c r="AF12" s="19">
+        <f>SUM(B12:AE12)</f>
+        <v>30</v>
       </c>
     </row>
-    <row r="13" ht="23" customHeight="1">
-      <c r="A13" s="17" t="inlineStr">
-        <is>
-          <t>Дежурных за день</t>
-        </is>
-      </c>
-      <c r="B13" s="18">
-        <f>COUNTIF(B5:B12,"+")</f>
-        <v>1</v>
-      </c>
-      <c r="C13" s="18">
-        <f>COUNTIF(C5:C12,"+")</f>
-        <v>1</v>
-      </c>
-      <c r="D13" s="18">
-        <f>COUNTIF(D5:D12,"+")</f>
-        <v>1</v>
-      </c>
-      <c r="E13" s="18">
-        <f>COUNTIF(E5:E12,"+")</f>
-        <v>1</v>
-      </c>
-      <c r="F13" s="18">
-        <f>COUNTIF(F5:F12,"+")</f>
-        <v>1</v>
-      </c>
-      <c r="G13" s="18">
-        <f>COUNTIF(G5:G12,"+")</f>
-        <v>1</v>
-      </c>
-      <c r="H13" s="18">
-        <f>COUNTIF(H5:H12,"+")</f>
-        <v>1</v>
-      </c>
-      <c r="I13" s="18">
-        <f>COUNTIF(I5:I12,"+")</f>
-        <v>1</v>
-      </c>
-      <c r="J13" s="18">
-        <f>COUNTIF(J5:J12,"+")</f>
-        <v>1</v>
-      </c>
-      <c r="K13" s="18">
-        <f>COUNTIF(K5:K12,"+")</f>
-        <v>1</v>
-      </c>
-      <c r="L13" s="18">
-        <f>COUNTIF(L5:L12,"+")</f>
-        <v>1</v>
-      </c>
-      <c r="M13" s="18">
-        <f>COUNTIF(M5:M12,"+")</f>
-        <v>1</v>
-      </c>
-      <c r="N13" s="18">
-        <f>COUNTIF(N5:N12,"+")</f>
-        <v>1</v>
-      </c>
-      <c r="O13" s="18">
-        <f>COUNTIF(O5:O12,"+")</f>
-        <v>1</v>
-      </c>
-      <c r="P13" s="18">
-        <f>COUNTIF(P5:P12,"+")</f>
-        <v>1</v>
-      </c>
-      <c r="Q13" s="18">
-        <f>COUNTIF(Q5:Q12,"+")</f>
-        <v>1</v>
-      </c>
-      <c r="R13" s="18">
-        <f>COUNTIF(R5:R12,"+")</f>
-        <v>1</v>
-      </c>
-      <c r="S13" s="18">
-        <f>COUNTIF(S5:S12,"+")</f>
-        <v>1</v>
-      </c>
-      <c r="T13" s="18">
-        <f>COUNTIF(T5:T12,"+")</f>
-        <v>1</v>
-      </c>
-      <c r="U13" s="18">
-        <f>COUNTIF(U5:U12,"+")</f>
-        <v>1</v>
-      </c>
-      <c r="V13" s="18">
-        <f>COUNTIF(V5:V12,"+")</f>
-        <v>1</v>
-      </c>
-      <c r="W13" s="18">
-        <f>COUNTIF(W5:W12,"+")</f>
-        <v>1</v>
-      </c>
-      <c r="X13" s="18">
-        <f>COUNTIF(X5:X12,"+")</f>
-        <v>1</v>
-      </c>
-      <c r="Y13" s="18">
-        <f>COUNTIF(Y5:Y12,"+")</f>
-        <v>1</v>
-      </c>
-      <c r="Z13" s="18">
-        <f>COUNTIF(Z5:Z12,"+")</f>
-        <v>1</v>
-      </c>
-      <c r="AA13" s="18">
-        <f>COUNTIF(AA5:AA12,"+")</f>
-        <v>1</v>
-      </c>
-      <c r="AB13" s="18">
-        <f>COUNTIF(AB5:AB12,"+")</f>
-        <v>1</v>
-      </c>
-      <c r="AC13" s="18">
-        <f>COUNTIF(AC5:AC12,"+")</f>
-        <v>1</v>
-      </c>
-      <c r="AD13" s="18">
-        <f>COUNTIF(AD5:AD12,"+")</f>
-        <v>1</v>
-      </c>
-      <c r="AE13" s="18">
-        <f>COUNTIF(AE5:AE12,"+")</f>
-        <v>1</v>
-      </c>
-      <c r="AF13" s="19">
-        <f>SUM(B13:AE13)</f>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="14" ht="7" customHeight="1"/>
+    <row r="13" ht="7" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:AF1"/>
@@ -1516,7 +1475,7 @@
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="AF3:AF4"/>
   </mergeCells>
-  <conditionalFormatting sqref="B13:AE13">
+  <conditionalFormatting sqref="B12:AE12">
     <cfRule type="cellIs" priority="1" operator="notEqual" dxfId="0">
       <formula>1</formula>
     </cfRule>

</xml_diff>